<commit_message>
Add client-facing Admin verification report (this round's brutal test pass)
Compiled the full "brutal test everything" round into a single PDF:
both original questions answered with live proof (all 3 return types
survive a real download-wipe-reupload round trip at 21/21; device
catalog scoping + the new "top N of M" message at 13/13), the full
panel-by-panel results table (139/139 checks across 10 suites), plain-
English writeups of the 4 real bugs found and fixed this round, the
one suspected bug investigated and ruled out, forward-looking risk
notes, and embedded screenshots as evidence throughout.

Refreshed the round-trip and device-catalog screenshots/downloads by
re-running both scripts to confirm current numbers before writing them
into the report.
</commit_message>
<xml_diff>
--- a/e2e-screenshots/return-types-round-trip/downloaded-sales-report.xlsx
+++ b/e2e-screenshots/return-types-round-trip/downloaded-sales-report.xlsx
@@ -177,43 +177,43 @@
     <t>Postage Loss</t>
   </si>
   <si>
+    <t>AMZ-2222</t>
+  </si>
+  <si>
+    <t>IP14-128-BLK</t>
+  </si>
+  <si>
+    <t>350190000092222</t>
+  </si>
+  <si>
+    <t>MOBILE WHOLESALE LTD</t>
+  </si>
+  <si>
+    <t>Refund</t>
+  </si>
+  <si>
+    <t>Refund — Faulty on arrival, RTS to supplier</t>
+  </si>
+  <si>
+    <t>AMZ-3333</t>
+  </si>
+  <si>
+    <t>350190000093333</t>
+  </si>
+  <si>
+    <t>In Repair</t>
+  </si>
+  <si>
+    <t>In Repair — Screen fault, needs bench repair</t>
+  </si>
+  <si>
     <t>AMZ-1111</t>
   </si>
   <si>
-    <t>IP14-128-BLK</t>
-  </si>
-  <si>
     <t>350190000091111</t>
   </si>
   <si>
-    <t>MOBILE WHOLESALE LTD</t>
-  </si>
-  <si>
-    <t>Refund</t>
-  </si>
-  <si>
     <t>Refund — Customer changed mind</t>
-  </si>
-  <si>
-    <t>AMZ-2222</t>
-  </si>
-  <si>
-    <t>350190000092222</t>
-  </si>
-  <si>
-    <t>Refund — Faulty on arrival, RTS to supplier</t>
-  </si>
-  <si>
-    <t>AMZ-3333</t>
-  </si>
-  <si>
-    <t>350190000093333</t>
-  </si>
-  <si>
-    <t>In Repair</t>
-  </si>
-  <si>
-    <t>In Repair — Screen fault, needs bench repair</t>
   </si>
   <si>
     <t>Customer Care Fees</t>
@@ -1347,10 +1347,10 @@
         <v>46230.5</v>
       </c>
       <c r="X3" s="8" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="Y3" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Z3" s="8">
         <v>2</v>
@@ -1367,13 +1367,13 @@
         <v>46213.5</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>53</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E4" s="8" t="s">
         <v>55</v>
@@ -1433,7 +1433,7 @@
         <v>46230.5</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="Y4" s="8" t="s">
         <v>64</v>
@@ -2098,7 +2098,7 @@
         <v>46230.5</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>103</v>
@@ -2148,7 +2148,7 @@
         <v>46230.5</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>103</v>
@@ -2198,7 +2198,7 @@
         <v>46230.5</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>103</v>
@@ -2222,10 +2222,10 @@
         <v>12</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L4" s="8" t="s">
         <v>111</v>
@@ -2279,7 +2279,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="B2" t="s">
         <v>103</v>
@@ -2302,7 +2302,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
         <v>103</v>
@@ -2325,7 +2325,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>103</v>
@@ -2348,7 +2348,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
         <v>103</v>
@@ -2371,7 +2371,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
         <v>103</v>
@@ -2394,7 +2394,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>103</v>
@@ -2417,7 +2417,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B8" t="s">
         <v>103</v>
@@ -2438,7 +2438,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B9" t="s">
         <v>103</v>
@@ -2461,7 +2461,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B10" t="s">
         <v>103</v>
@@ -2484,7 +2484,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>103</v>
@@ -2507,7 +2507,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
         <v>103</v>
@@ -2519,7 +2519,7 @@
         <v>123</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" t="s">

</xml_diff>

<commit_message>
Refresh more E2E evidence from the ongoing full-suite sweep
</commit_message>
<xml_diff>
--- a/e2e-screenshots/return-types-round-trip/downloaded-sales-report.xlsx
+++ b/e2e-screenshots/return-types-round-trip/downloaded-sales-report.xlsx
@@ -177,21 +177,30 @@
     <t>Postage Loss</t>
   </si>
   <si>
+    <t>AMZ-1111</t>
+  </si>
+  <si>
+    <t>IP14-128-BLK</t>
+  </si>
+  <si>
+    <t>350190000091111</t>
+  </si>
+  <si>
+    <t>MOBILE WHOLESALE LTD</t>
+  </si>
+  <si>
+    <t>Refund</t>
+  </si>
+  <si>
+    <t>Refund — Customer changed mind</t>
+  </si>
+  <si>
     <t>AMZ-2222</t>
   </si>
   <si>
-    <t>IP14-128-BLK</t>
-  </si>
-  <si>
     <t>350190000092222</t>
   </si>
   <si>
-    <t>MOBILE WHOLESALE LTD</t>
-  </si>
-  <si>
-    <t>Refund</t>
-  </si>
-  <si>
     <t>Refund — Faulty on arrival, RTS to supplier</t>
   </si>
   <si>
@@ -205,15 +214,6 @@
   </si>
   <si>
     <t>In Repair — Screen fault, needs bench repair</t>
-  </si>
-  <si>
-    <t>AMZ-1111</t>
-  </si>
-  <si>
-    <t>350190000091111</t>
-  </si>
-  <si>
-    <t>Refund — Customer changed mind</t>
   </si>
   <si>
     <t>Customer Care Fees</t>
@@ -1347,10 +1347,10 @@
         <v>46230.5</v>
       </c>
       <c r="X3" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y3" s="8" t="s">
         <v>60</v>
-      </c>
-      <c r="Y3" s="8" t="s">
-        <v>61</v>
       </c>
       <c r="Z3" s="8">
         <v>2</v>
@@ -1367,13 +1367,13 @@
         <v>46213.5</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>53</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E4" s="8" t="s">
         <v>55</v>
@@ -1433,7 +1433,7 @@
         <v>46230.5</v>
       </c>
       <c r="X4" s="8" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="Y4" s="8" t="s">
         <v>64</v>
@@ -2098,7 +2098,7 @@
         <v>46230.5</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>103</v>
@@ -2148,7 +2148,7 @@
         <v>46230.5</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>103</v>
@@ -2198,7 +2198,7 @@
         <v>46230.5</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>103</v>
@@ -2222,10 +2222,10 @@
         <v>12</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="L4" s="8" t="s">
         <v>111</v>
@@ -2279,7 +2279,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
         <v>103</v>
@@ -2302,7 +2302,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
         <v>103</v>
@@ -2325,7 +2325,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>103</v>
@@ -2348,7 +2348,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B5" t="s">
         <v>103</v>
@@ -2371,7 +2371,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B6" t="s">
         <v>103</v>
@@ -2394,7 +2394,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>103</v>
@@ -2417,7 +2417,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B8" t="s">
         <v>103</v>
@@ -2438,7 +2438,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B9" t="s">
         <v>103</v>
@@ -2461,7 +2461,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B10" t="s">
         <v>103</v>
@@ -2484,7 +2484,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>103</v>
@@ -2507,7 +2507,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B12" t="s">
         <v>103</v>
@@ -2519,7 +2519,7 @@
         <v>123</v>
       </c>
       <c r="E12" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" t="s">

</xml_diff>